<commit_message>
auto: sync changes 2026-06-02 12:43:19
</commit_message>
<xml_diff>
--- a/projects/Template.xlsx
+++ b/projects/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Copilot\RND-Dashboard\projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE904DC-D761-46B0-A963-9723FE618765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02680C2D-AC28-402B-96B9-98A796977D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B8D78CEB-D3AC-4A62-AA68-81CAD437EBFB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B8D78CEB-D3AC-4A62-AA68-81CAD437EBFB}"/>
   </bookViews>
   <sheets>
     <sheet name="개요" sheetId="1" r:id="rId1"/>
@@ -1305,6 +1305,39 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="6" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1312,39 +1345,6 @@
     <xf numFmtId="41" fontId="6" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1893,7 +1893,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="Z4" s="2">
-        <f>사업비!M4*0.4</f>
+        <f>개요!M19*0.4</f>
         <v>0</v>
       </c>
     </row>
@@ -2042,51 +2042,311 @@
       <c r="E15" s="30"/>
       <c r="H15" s="23"/>
     </row>
-    <row r="16" spans="1:27" ht="15" customHeight="1">
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="30"/>
-      <c r="H16" s="23"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-      <c r="V16" s="4"/>
-      <c r="W16" s="4"/>
-    </row>
-    <row r="17" spans="2:23" ht="15" customHeight="1">
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="30"/>
-      <c r="H17" s="23"/>
-    </row>
-    <row r="20" spans="2:23" s="4" customFormat="1" ht="15" customHeight="1">
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="2"/>
-      <c r="W20" s="2"/>
-    </row>
-    <row r="27" spans="2:23" ht="15" customHeight="1">
+    <row r="16" spans="1:27" customFormat="1" ht="21.6">
+      <c r="A16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="M16" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="N16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="O16" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="50" t="str">
+        <f>IF(B17="","",DATEDIF(B17,C17,"m")+1)</f>
+        <v/>
+      </c>
+      <c r="E17" s="80" cm="1">
+        <f t="array" ref="E17">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K17) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="70"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="71"/>
+      <c r="I17" s="43"/>
+      <c r="J17" s="60">
+        <f>H17+I17</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="61">
+        <f>SUM(F17,G17,H17)</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="61">
+        <f>I17</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="62">
+        <f>K17+L17</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="16"/>
+      <c r="O17" s="72"/>
+    </row>
+    <row r="18" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A18" s="73"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="51" t="str">
+        <f>IF(B18="","",DATEDIF(B18,C18,"m")+1)</f>
+        <v/>
+      </c>
+      <c r="E18" s="65" cm="1">
+        <f t="array" ref="E18">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K18) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="74"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="76"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="63">
+        <f>H18+I18</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="64">
+        <f>SUM(F18,G18,H18)</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="65">
+        <f>I18</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="66">
+        <f>K18+L18</f>
+        <v>0</v>
+      </c>
+      <c r="N18" s="77"/>
+      <c r="O18" s="78"/>
+    </row>
+    <row r="19" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="50" t="str">
+        <f>IF(B19="","",DATEDIF(B19,C19,"m")+1)</f>
+        <v/>
+      </c>
+      <c r="E19" s="80" cm="1">
+        <f t="array" ref="E19">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K19) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="70"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="71"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="60">
+        <f>H19+I19</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="61">
+        <f>SUM(F19,G19,H19)</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="61">
+        <f>I19</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="62">
+        <f>K19+L19</f>
+        <v>0</v>
+      </c>
+      <c r="N19" s="16"/>
+      <c r="O19" s="72"/>
+    </row>
+    <row r="20" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A20" s="73"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="51" t="str">
+        <f>IF(B20="","",DATEDIF(B20,C20,"m")+1)</f>
+        <v/>
+      </c>
+      <c r="E20" s="65" cm="1">
+        <f t="array" ref="E20">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K20) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="74"/>
+      <c r="G20" s="75"/>
+      <c r="H20" s="79"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="67">
+        <f>H20+I20</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="64">
+        <f>SUM(F20,G20,H20)</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="65">
+        <f>I20</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="66">
+        <f>K20+L20</f>
+        <v>0</v>
+      </c>
+      <c r="N20" s="77"/>
+      <c r="O20" s="78"/>
+    </row>
+    <row r="21" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A21" s="45"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="50" t="str">
+        <f>IF(B21="","",DATEDIF(B21,C21,"m")+1)</f>
+        <v/>
+      </c>
+      <c r="E21" s="80" cm="1">
+        <f t="array" ref="E21">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K21) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="46"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="68">
+        <f>H21+I21</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="69">
+        <f>SUM(F21,G21,H21)</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="61">
+        <f>I21</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="62">
+        <f>K21+L21</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="16"/>
+      <c r="O21" s="72"/>
+    </row>
+    <row r="22" spans="1:15" customFormat="1" ht="17.399999999999999">
+      <c r="A22" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="52">
+        <f>SUM(D17:D21)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="53" cm="1">
+        <f t="array" ref="E22">SUMPRODUCT(
+  (사업비!$A$17:$A$51 = $K22) *
+  ISNUMBER(MATCH(사업비!$B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
+  사업비!$C$17:$C$51
+)</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="54">
+        <f>SUM(F17:F21)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="52">
+        <f>SUM(G17:G21)</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="55">
+        <f>SUM(H17:H21)</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="56">
+        <f>SUM(I17:I21)</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="57">
+        <f>SUM(J17:J21)</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="58">
+        <f>SUM(K17:K21)</f>
+        <v>0</v>
+      </c>
+      <c r="L22" s="58">
+        <f>SUM(L17:L21)</f>
+        <v>0</v>
+      </c>
+      <c r="M22" s="59">
+        <f>SUM(M17:M21)</f>
+        <v>0</v>
+      </c>
+      <c r="N22" s="59">
+        <f>SUM(N17:N21)</f>
+        <v>0</v>
+      </c>
+      <c r="O22" s="81">
+        <f>SUM(O17:O21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="15" customHeight="1">
       <c r="C27" s="31"/>
     </row>
-    <row r="28" spans="2:23" ht="15" customHeight="1">
+    <row r="28" spans="1:15" ht="15" customHeight="1">
       <c r="B28" s="24"/>
       <c r="C28" s="31"/>
       <c r="D28" s="31"/>
@@ -2126,7 +2386,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F547BFE0-1680-4D6E-87BD-0997B5AC0514}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
     <col min="5" max="5" width="7.3984375" bestFit="1" customWidth="1"/>
@@ -2134,315 +2394,9 @@
     <col min="12" max="12" width="8.69921875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.69921875" bestFit="1" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:15" ht="21.6">
-      <c r="A1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="O1" s="13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="50" t="str">
-        <f>IF(B2="","",DATEDIF(B2,C2,"m")+1)</f>
-        <v/>
-      </c>
-      <c r="E2" s="80" cm="1">
-        <f t="array" ref="E2">SUMPRODUCT(
-  ($A$17:$A$51 = $K2) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="60">
-        <f>H2+I2</f>
-        <v>0</v>
-      </c>
-      <c r="K2" s="61">
-        <f>SUM(F2,G2,H2)</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="61">
-        <f>I2</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="62">
-        <f>K2+L2</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="72"/>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="73"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="51" t="str">
-        <f t="shared" ref="D3:D4" si="0">IF(B3="","",DATEDIF(B3,C3,"m")+1)</f>
-        <v/>
-      </c>
-      <c r="E3" s="65" cm="1">
-        <f t="array" ref="E3">SUMPRODUCT(
-  ($A$17:$A$51 = $K3) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="74"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="63">
-        <f t="shared" ref="J3:J6" si="1">H3+I3</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="64">
-        <f t="shared" ref="K3:K5" si="2">SUM(F3,G3,H3)</f>
-        <v>0</v>
-      </c>
-      <c r="L3" s="65">
-        <f t="shared" ref="L3:L6" si="3">I3</f>
-        <v>0</v>
-      </c>
-      <c r="M3" s="66">
-        <f>K3+L3</f>
-        <v>0</v>
-      </c>
-      <c r="N3" s="77"/>
-      <c r="O3" s="78"/>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="14"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="50" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E4" s="80" cm="1">
-        <f t="array" ref="E4">SUMPRODUCT(
-  ($A$17:$A$51 = $K4) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="70"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="71"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="60">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K4" s="61">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L4" s="61">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M4" s="62">
-        <f t="shared" ref="M4:M6" si="4">K4+L4</f>
-        <v>0</v>
-      </c>
-      <c r="N4" s="16"/>
-      <c r="O4" s="72"/>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="73"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="51" t="str">
-        <f>IF(B5="","",DATEDIF(B5,C5,"m")+1)</f>
-        <v/>
-      </c>
-      <c r="E5" s="65" cm="1">
-        <f t="array" ref="E5">SUMPRODUCT(
-  ($A$17:$A$51 = $K5) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="74"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="79"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="67">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K5" s="64">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L5" s="65">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M5" s="66">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N5" s="77"/>
-      <c r="O5" s="78"/>
-    </row>
-    <row r="6" spans="1:15">
-      <c r="A6" s="45"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="50" t="str">
-        <f t="shared" ref="D6" si="5">IF(B6="","",DATEDIF(B6,C6,"m")+1)</f>
-        <v/>
-      </c>
-      <c r="E6" s="80" cm="1">
-        <f t="array" ref="E6">SUMPRODUCT(
-  ($A$17:$A$51 = $K6) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="46"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="68">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="69">
-        <f>SUM(F6,G6,H6)</f>
-        <v>0</v>
-      </c>
-      <c r="L6" s="61">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M6" s="62">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="72"/>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="52">
-        <f t="shared" ref="D7" si="6">SUM(D2:D6)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="53" cm="1">
-        <f t="array" ref="E7">SUMPRODUCT(
-  ($A$17:$A$51 = $K7) *
-  ISNUMBER(MATCH($B$17:$B$51, {"인건비","연구활동비","연구재료비","연구시설장비비","연구수당"}, 0)) *
-  $C$17:$C$51
-)</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="54">
-        <f>SUM(F2:F6)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="52">
-        <f>SUM(G2:G6)</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="55">
-        <f>SUM(H2:H6)</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="56">
-        <f>SUM(I2:I6)</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="57">
-        <f t="shared" ref="J7:K7" si="7">SUM(J2:J6)</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="58">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="L7" s="58">
-        <f>SUM(L2:L6)</f>
-        <v>0</v>
-      </c>
-      <c r="M7" s="59">
-        <f t="shared" ref="M7" si="8">SUM(M2:M6)</f>
-        <v>0</v>
-      </c>
-      <c r="N7" s="59">
-        <f>SUM(N2:N6)</f>
-        <v>0</v>
-      </c>
-      <c r="O7" s="81">
-        <f>SUM(O2:O6)</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <sheetData/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="D6:M6 D7 E7:M7 N7:O7 D2:E2 J2:M2 D3:E5 J3:M5 G2 G3:G5" unlockedFormula="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -2459,14 +2413,14 @@
       <c r="A1" s="33"/>
       <c r="B1" s="37"/>
       <c r="C1" s="33"/>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="100" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="89"/>
-      <c r="F1" s="90" t="s">
+      <c r="E1" s="100"/>
+      <c r="F1" s="101" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="90"/>
+      <c r="G1" s="101"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="34" t="s">
@@ -3089,7 +3043,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C4C0AB1B-468E-4B95-9E28-23CEE24A29DF}">
           <x14:formula1>
-            <xm:f>사업비!$A$2:$A$6</xm:f>
+            <xm:f>개요!$A$17:$A$21</xm:f>
           </x14:formula1>
           <xm:sqref>C3:C50</xm:sqref>
         </x14:dataValidation>
@@ -3104,74 +3058,74 @@
   <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="54.59765625" style="92" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="54.59765625" style="90" bestFit="1" customWidth="1"/>
     <col min="2" max="16384" width="8.796875" style="82"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.399999999999999" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="94" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="93" t="s">
+      <c r="C1" s="94" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="93" t="s">
+      <c r="D1" s="94" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="94" t="s">
+      <c r="E1" s="97" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="95"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="94" t="s">
+      <c r="F1" s="98"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="95"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="97" t="s">
+      <c r="I1" s="98"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="96" t="s">
         <v>39</v>
       </c>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="98"/>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="99" t="s">
+      <c r="A2" s="95"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="91" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="99" t="s">
+      <c r="F2" s="91" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="99" t="s">
+      <c r="G2" s="91" t="s">
         <v>45</v>
       </c>
-      <c r="H2" s="99" t="s">
+      <c r="H2" s="91" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="99" t="s">
+      <c r="I2" s="91" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="99" t="s">
+      <c r="J2" s="91" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="99" t="s">
+      <c r="K2" s="91" t="s">
         <v>46</v>
       </c>
-      <c r="L2" s="99" t="s">
+      <c r="L2" s="91" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="99" t="s">
+      <c r="M2" s="91" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="91"/>
+      <c r="A3" s="89"/>
       <c r="B3" s="83"/>
       <c r="C3" s="83"/>
       <c r="D3" s="83"/>
@@ -3215,7 +3169,7 @@
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="91"/>
+      <c r="A4" s="89"/>
       <c r="B4" s="83"/>
       <c r="C4" s="83"/>
       <c r="D4" s="83"/>
@@ -3254,7 +3208,7 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="91"/>
+      <c r="A5" s="89"/>
       <c r="B5" s="83"/>
       <c r="C5" s="83"/>
       <c r="D5" s="83"/>
@@ -3293,7 +3247,7 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="91"/>
+      <c r="A6" s="89"/>
       <c r="B6" s="83"/>
       <c r="C6" s="83"/>
       <c r="D6" s="83"/>
@@ -3332,7 +3286,7 @@
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="91"/>
+      <c r="A7" s="89"/>
       <c r="B7" s="83"/>
       <c r="C7" s="83"/>
       <c r="D7" s="83"/>
@@ -3371,7 +3325,7 @@
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="91"/>
+      <c r="A8" s="89"/>
       <c r="B8" s="83"/>
       <c r="C8" s="83"/>
       <c r="D8" s="83"/>
@@ -3410,7 +3364,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="91"/>
+      <c r="A9" s="89"/>
       <c r="B9" s="83"/>
       <c r="C9" s="83"/>
       <c r="D9" s="83"/>
@@ -3449,7 +3403,7 @@
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="91"/>
+      <c r="A10" s="89"/>
       <c r="B10" s="83"/>
       <c r="C10" s="83"/>
       <c r="D10" s="83"/>
@@ -3488,7 +3442,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="91"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="83"/>
       <c r="C11" s="83"/>
       <c r="D11" s="83"/>
@@ -3527,7 +3481,7 @@
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="91"/>
+      <c r="A12" s="89"/>
       <c r="B12" s="83"/>
       <c r="C12" s="83"/>
       <c r="D12" s="83"/>
@@ -3566,7 +3520,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="91"/>
+      <c r="A13" s="89"/>
       <c r="B13" s="83"/>
       <c r="C13" s="83"/>
       <c r="D13" s="83"/>
@@ -3605,7 +3559,7 @@
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="91"/>
+      <c r="A14" s="89"/>
       <c r="B14" s="83"/>
       <c r="C14" s="83"/>
       <c r="D14" s="83"/>
@@ -3635,7 +3589,7 @@
       <c r="M14" s="85"/>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="91"/>
+      <c r="A15" s="89"/>
       <c r="B15" s="83"/>
       <c r="C15" s="83"/>
       <c r="D15" s="83"/>
@@ -3665,7 +3619,7 @@
       <c r="M15" s="85"/>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="91"/>
+      <c r="A16" s="89"/>
       <c r="B16" s="83"/>
       <c r="C16" s="83"/>
       <c r="D16" s="83"/>
@@ -3695,7 +3649,7 @@
       <c r="M16" s="85"/>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="91"/>
+      <c r="A17" s="89"/>
       <c r="B17" s="83"/>
       <c r="C17" s="83"/>
       <c r="D17" s="83"/>
@@ -3725,7 +3679,7 @@
       <c r="M17" s="85"/>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="91"/>
+      <c r="A18" s="89"/>
       <c r="B18" s="83"/>
       <c r="C18" s="83"/>
       <c r="D18" s="83"/>
@@ -3755,7 +3709,7 @@
       <c r="M18" s="85"/>
     </row>
     <row r="19" spans="1:13">
-      <c r="A19" s="91"/>
+      <c r="A19" s="89"/>
       <c r="B19" s="83"/>
       <c r="C19" s="83"/>
       <c r="D19" s="83"/>
@@ -3785,7 +3739,7 @@
       <c r="M19" s="85"/>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" s="91"/>
+      <c r="A20" s="89"/>
       <c r="B20" s="83"/>
       <c r="C20" s="83"/>
       <c r="D20" s="83"/>
@@ -3815,7 +3769,7 @@
       <c r="M20" s="85"/>
     </row>
     <row r="21" spans="1:13">
-      <c r="A21" s="91"/>
+      <c r="A21" s="89"/>
       <c r="B21" s="83"/>
       <c r="C21" s="83"/>
       <c r="D21" s="83"/>
@@ -3854,7 +3808,7 @@
       </c>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" s="91"/>
+      <c r="A22" s="89"/>
       <c r="B22" s="83"/>
       <c r="C22" s="83"/>
       <c r="D22" s="83"/>
@@ -3893,7 +3847,7 @@
       </c>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" s="91"/>
+      <c r="A23" s="89"/>
       <c r="B23" s="83"/>
       <c r="C23" s="83"/>
       <c r="D23" s="83"/>
@@ -3923,7 +3877,7 @@
       <c r="M23" s="85"/>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" s="91"/>
+      <c r="A24" s="89"/>
       <c r="B24" s="83"/>
       <c r="C24" s="83"/>
       <c r="D24" s="83"/>
@@ -3953,7 +3907,7 @@
       <c r="M24" s="85"/>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="91"/>
+      <c r="A25" s="89"/>
       <c r="B25" s="83"/>
       <c r="C25" s="83"/>
       <c r="D25" s="83"/>
@@ -3983,7 +3937,7 @@
       <c r="M25" s="85"/>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" s="91"/>
+      <c r="A26" s="89"/>
       <c r="B26" s="83"/>
       <c r="C26" s="83"/>
       <c r="D26" s="83"/>
@@ -4013,7 +3967,7 @@
       <c r="M26" s="85"/>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="91"/>
+      <c r="A27" s="89"/>
       <c r="B27" s="83"/>
       <c r="C27" s="83"/>
       <c r="D27" s="83"/>
@@ -4052,7 +4006,7 @@
       </c>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="91"/>
+      <c r="A28" s="89"/>
       <c r="B28" s="83"/>
       <c r="C28" s="83"/>
       <c r="D28" s="83"/>
@@ -4091,7 +4045,7 @@
       </c>
     </row>
     <row r="29" spans="1:13">
-      <c r="A29" s="91"/>
+      <c r="A29" s="89"/>
       <c r="B29" s="83"/>
       <c r="C29" s="83"/>
       <c r="D29" s="83"/>
@@ -4130,7 +4084,7 @@
       </c>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="91"/>
+      <c r="A30" s="89"/>
       <c r="B30" s="83"/>
       <c r="C30" s="83"/>
       <c r="D30" s="83"/>
@@ -4169,7 +4123,7 @@
       </c>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="91" t="s">
+      <c r="A31" s="89" t="s">
         <v>40</v>
       </c>
       <c r="B31" s="83"/>
@@ -4237,7 +4191,7 @@
   <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="10.8"/>
   <cols>
-    <col min="1" max="1" width="54.59765625" style="101" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="54.59765625" style="93" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.296875" style="88" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.09765625" style="88" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.5" style="88" bestFit="1" customWidth="1"/>
@@ -4259,295 +4213,295 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A2" s="100"/>
+      <c r="A2" s="92"/>
       <c r="B2" s="86"/>
       <c r="C2" s="86"/>
       <c r="D2" s="86"/>
     </row>
     <row r="3" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A3" s="100"/>
+      <c r="A3" s="92"/>
       <c r="B3" s="86"/>
       <c r="C3" s="86"/>
       <c r="D3" s="86"/>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A4" s="100"/>
+      <c r="A4" s="92"/>
       <c r="B4" s="86"/>
       <c r="C4" s="86"/>
       <c r="D4" s="86"/>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A5" s="100"/>
+      <c r="A5" s="92"/>
       <c r="B5" s="86"/>
       <c r="C5" s="86"/>
       <c r="D5" s="86"/>
     </row>
     <row r="6" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A6" s="100"/>
+      <c r="A6" s="92"/>
       <c r="B6" s="86"/>
       <c r="C6" s="86"/>
       <c r="D6" s="86"/>
     </row>
     <row r="7" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A7" s="100"/>
+      <c r="A7" s="92"/>
       <c r="B7" s="86"/>
       <c r="C7" s="86"/>
       <c r="D7" s="86"/>
     </row>
     <row r="8" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A8" s="100"/>
+      <c r="A8" s="92"/>
       <c r="B8" s="86"/>
       <c r="C8" s="86"/>
       <c r="D8" s="86"/>
     </row>
     <row r="9" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A9" s="100"/>
+      <c r="A9" s="92"/>
       <c r="B9" s="86"/>
       <c r="C9" s="86"/>
       <c r="D9" s="86"/>
     </row>
     <row r="10" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A10" s="100"/>
+      <c r="A10" s="92"/>
       <c r="B10" s="86"/>
       <c r="C10" s="86"/>
       <c r="D10" s="86"/>
     </row>
     <row r="11" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A11" s="100"/>
+      <c r="A11" s="92"/>
       <c r="B11" s="86"/>
       <c r="C11" s="86"/>
       <c r="D11" s="86"/>
     </row>
     <row r="12" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A12" s="100"/>
+      <c r="A12" s="92"/>
       <c r="B12" s="86"/>
       <c r="C12" s="86"/>
       <c r="D12" s="86"/>
     </row>
     <row r="13" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A13" s="100"/>
+      <c r="A13" s="92"/>
       <c r="B13" s="86"/>
       <c r="C13" s="86"/>
       <c r="D13" s="86"/>
     </row>
     <row r="14" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A14" s="100"/>
+      <c r="A14" s="92"/>
       <c r="B14" s="86"/>
       <c r="C14" s="86"/>
       <c r="D14" s="86"/>
     </row>
     <row r="15" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A15" s="100"/>
+      <c r="A15" s="92"/>
       <c r="B15" s="86"/>
       <c r="C15" s="86"/>
       <c r="D15" s="86"/>
     </row>
     <row r="16" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A16" s="100"/>
+      <c r="A16" s="92"/>
       <c r="B16" s="86"/>
       <c r="C16" s="86"/>
       <c r="D16" s="86"/>
     </row>
     <row r="17" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A17" s="100"/>
+      <c r="A17" s="92"/>
       <c r="B17" s="86"/>
       <c r="C17" s="86"/>
       <c r="D17" s="86"/>
     </row>
     <row r="18" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A18" s="100"/>
+      <c r="A18" s="92"/>
       <c r="B18" s="86"/>
       <c r="C18" s="86"/>
       <c r="D18" s="86"/>
     </row>
     <row r="19" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A19" s="100"/>
+      <c r="A19" s="92"/>
       <c r="B19" s="86"/>
       <c r="C19" s="86"/>
       <c r="D19" s="86"/>
     </row>
     <row r="20" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A20" s="100"/>
+      <c r="A20" s="92"/>
       <c r="B20" s="86"/>
       <c r="C20" s="86"/>
       <c r="D20" s="86"/>
     </row>
     <row r="21" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A21" s="100"/>
+      <c r="A21" s="92"/>
       <c r="B21" s="86"/>
       <c r="C21" s="86"/>
       <c r="D21" s="86"/>
     </row>
     <row r="22" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A22" s="100"/>
+      <c r="A22" s="92"/>
       <c r="B22" s="86"/>
       <c r="C22" s="86"/>
       <c r="D22" s="86"/>
     </row>
     <row r="23" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A23" s="100"/>
+      <c r="A23" s="92"/>
       <c r="B23" s="86"/>
       <c r="C23" s="86"/>
       <c r="D23" s="86"/>
     </row>
     <row r="24" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A24" s="100"/>
+      <c r="A24" s="92"/>
       <c r="B24" s="86"/>
       <c r="C24" s="86"/>
       <c r="D24" s="86"/>
     </row>
     <row r="25" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A25" s="100"/>
+      <c r="A25" s="92"/>
       <c r="B25" s="86"/>
       <c r="C25" s="86"/>
       <c r="D25" s="86"/>
     </row>
     <row r="26" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A26" s="100"/>
+      <c r="A26" s="92"/>
       <c r="B26" s="86"/>
       <c r="C26" s="86"/>
       <c r="D26" s="86"/>
     </row>
     <row r="27" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A27" s="100"/>
+      <c r="A27" s="92"/>
       <c r="B27" s="86"/>
       <c r="C27" s="86"/>
       <c r="D27" s="86"/>
     </row>
     <row r="28" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A28" s="100"/>
+      <c r="A28" s="92"/>
       <c r="B28" s="86"/>
       <c r="C28" s="86"/>
       <c r="D28" s="86"/>
     </row>
     <row r="29" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A29" s="100"/>
+      <c r="A29" s="92"/>
       <c r="B29" s="86"/>
       <c r="C29" s="86"/>
       <c r="D29" s="86"/>
     </row>
     <row r="30" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A30" s="100"/>
+      <c r="A30" s="92"/>
       <c r="B30" s="86"/>
       <c r="C30" s="86"/>
       <c r="D30" s="86"/>
     </row>
     <row r="31" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A31" s="100"/>
+      <c r="A31" s="92"/>
       <c r="B31" s="86"/>
       <c r="C31" s="86"/>
       <c r="D31" s="86"/>
     </row>
     <row r="32" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A32" s="100"/>
+      <c r="A32" s="92"/>
       <c r="B32" s="86"/>
       <c r="C32" s="86"/>
       <c r="D32" s="86"/>
     </row>
     <row r="33" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A33" s="100"/>
+      <c r="A33" s="92"/>
       <c r="B33" s="86"/>
       <c r="C33" s="86"/>
       <c r="D33" s="86"/>
     </row>
     <row r="34" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A34" s="100"/>
+      <c r="A34" s="92"/>
       <c r="B34" s="86"/>
       <c r="C34" s="86"/>
       <c r="D34" s="86"/>
     </row>
     <row r="35" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A35" s="100"/>
+      <c r="A35" s="92"/>
       <c r="B35" s="86"/>
       <c r="C35" s="86"/>
       <c r="D35" s="86"/>
     </row>
     <row r="36" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A36" s="100"/>
+      <c r="A36" s="92"/>
       <c r="B36" s="86"/>
       <c r="C36" s="86"/>
       <c r="D36" s="86"/>
     </row>
     <row r="37" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A37" s="100"/>
+      <c r="A37" s="92"/>
       <c r="B37" s="86"/>
       <c r="C37" s="86"/>
       <c r="D37" s="86"/>
     </row>
     <row r="38" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A38" s="100"/>
+      <c r="A38" s="92"/>
       <c r="B38" s="86"/>
       <c r="C38" s="86"/>
       <c r="D38" s="86"/>
     </row>
     <row r="39" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A39" s="100"/>
+      <c r="A39" s="92"/>
       <c r="B39" s="86"/>
       <c r="C39" s="86"/>
       <c r="D39" s="86"/>
     </row>
     <row r="40" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A40" s="100"/>
+      <c r="A40" s="92"/>
       <c r="B40" s="86"/>
       <c r="C40" s="86"/>
       <c r="D40" s="86"/>
     </row>
     <row r="41" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A41" s="100"/>
+      <c r="A41" s="92"/>
       <c r="B41" s="86"/>
       <c r="C41" s="86"/>
       <c r="D41" s="86"/>
     </row>
     <row r="42" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A42" s="100"/>
+      <c r="A42" s="92"/>
       <c r="B42" s="86"/>
       <c r="C42" s="86"/>
       <c r="D42" s="86"/>
     </row>
     <row r="43" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A43" s="100"/>
+      <c r="A43" s="92"/>
       <c r="B43" s="86"/>
       <c r="C43" s="86"/>
       <c r="D43" s="86"/>
     </row>
     <row r="44" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A44" s="100"/>
+      <c r="A44" s="92"/>
       <c r="B44" s="86"/>
       <c r="C44" s="86"/>
       <c r="D44" s="86"/>
     </row>
     <row r="45" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A45" s="100"/>
+      <c r="A45" s="92"/>
       <c r="B45" s="86"/>
       <c r="C45" s="86"/>
       <c r="D45" s="86"/>
     </row>
     <row r="46" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A46" s="100"/>
+      <c r="A46" s="92"/>
       <c r="B46" s="86"/>
       <c r="C46" s="86"/>
       <c r="D46" s="86"/>
     </row>
     <row r="47" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A47" s="100"/>
+      <c r="A47" s="92"/>
       <c r="B47" s="86"/>
       <c r="C47" s="86"/>
       <c r="D47" s="86"/>
     </row>
     <row r="48" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A48" s="100"/>
+      <c r="A48" s="92"/>
       <c r="B48" s="86"/>
       <c r="C48" s="86"/>
       <c r="D48" s="86"/>
     </row>
     <row r="49" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A49" s="100"/>
+      <c r="A49" s="92"/>
       <c r="B49" s="86"/>
       <c r="C49" s="86"/>
       <c r="D49" s="86"/>
     </row>
     <row r="50" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A50" s="100"/>
+      <c r="A50" s="92"/>
       <c r="B50" s="86"/>
       <c r="C50" s="86"/>
       <c r="D50" s="86"/>
@@ -4579,17 +4533,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7F1AA64A-1E17-4A37-91B7-C07A673F52E3}">
-          <x14:formula1>
-            <xm:f>사업비!$A$2:$A$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2:B24</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{940C646E-5367-4D64-81B5-92B0C3F2072A}">
           <x14:formula1>
             <xm:f>정량지표!$A$3:$A$30</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A32</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7F1AA64A-1E17-4A37-91B7-C07A673F52E3}">
+          <x14:formula1>
+            <xm:f>개요!$A$17:$A$21</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B24</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>